<commit_message>
Complete excel Clean project
</commit_message>
<xml_diff>
--- a/Client_Transactions.xlsx
+++ b/Client_Transactions.xlsx
@@ -8,12 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\1.My_Project\Excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EF3DA749-9BAB-4156-ACE4-AE0FD56D08A4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A7D3E174-A676-40B4-8D6A-06F0BDFC9DCA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="372" windowWidth="23256" windowHeight="12696" xr2:uid="{7F7E1DDE-3781-814A-825E-072C922D74F6}"/>
+    <workbookView xWindow="-108" yWindow="372" windowWidth="23256" windowHeight="12696" activeTab="2" xr2:uid="{7F7E1DDE-3781-814A-825E-072C922D74F6}"/>
   </bookViews>
   <sheets>
-    <sheet name="Data" sheetId="2" r:id="rId1"/>
+    <sheet name="Original_Data" sheetId="3" r:id="rId1"/>
+    <sheet name="Cleand_Data" sheetId="2" r:id="rId2"/>
+    <sheet name="Steps" sheetId="4" r:id="rId3"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -36,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="130" uniqueCount="72">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="315" uniqueCount="167">
   <si>
     <t>Date</t>
   </si>
@@ -59,6 +61,90 @@
     <t>Department</t>
   </si>
   <si>
+    <t>AMAZON.COM, INC. (XNAS:AMZN)</t>
+  </si>
+  <si>
+    <t>TESLA, INC. (XNAS:TSLA)</t>
+  </si>
+  <si>
+    <t>NETFLIX, INC. (XNAS:NFLX)</t>
+  </si>
+  <si>
+    <t>THE PROCTER &amp; GAMBLE COMPANY (XNYS:PG)</t>
+  </si>
+  <si>
+    <t>THE GOLDMAN SACHS GROUP, INC. (XNYS:GS)</t>
+  </si>
+  <si>
+    <t>JPMORGAN CHASE &amp; CO. (XNYS:JPM)</t>
+  </si>
+  <si>
+    <t>MORGAN STANLEY (XNYS:MS)</t>
+  </si>
+  <si>
+    <t>CITIGROUP INC. (XNYS:C)</t>
+  </si>
+  <si>
+    <t>BANK OF AMERICA CORPORATION (XNYS:BAC)</t>
+  </si>
+  <si>
+    <t>WALMART INC. (XNYS:WMT)</t>
+  </si>
+  <si>
+    <t>TARGET CORPORATION (XNYS:TGT)</t>
+  </si>
+  <si>
+    <t>COSTCO WHOLESALE CORPORATION (XNAS:COST)</t>
+  </si>
+  <si>
+    <t>MCDONALD'S CORPORATION (XNYS:MCD)</t>
+  </si>
+  <si>
+    <t>EXXON MOBIL CORPORATION (XNYS:XOM)</t>
+  </si>
+  <si>
+    <t>VERIZON COMMUNICATIONS INC. (XNYS:VZ)</t>
+  </si>
+  <si>
+    <t>THE HOME DEPOT, INC. (XNYS:HD)</t>
+  </si>
+  <si>
+    <t>CISCO SYSTEMS, INC. (XNAS:CSCO)</t>
+  </si>
+  <si>
+    <t>CHEVRON CORPORATION (XNYS:CVX)</t>
+  </si>
+  <si>
+    <t>AT&amp;T INC. (XNYS:T)</t>
+  </si>
+  <si>
+    <t>INTEL CORPORATION (XNAS:INTC)</t>
+  </si>
+  <si>
+    <t>GENERAL MOTORS COMPANY (XNYS:GM)</t>
+  </si>
+  <si>
+    <t>MICROSOFT CORPORATION (XNAS:MSFT)</t>
+  </si>
+  <si>
+    <t>COMCAST CORPORATION (XNAS:CMCSA)</t>
+  </si>
+  <si>
+    <t>DELL TECHNOLOGIES INC. (XNYS:DELL)</t>
+  </si>
+  <si>
+    <t>JOHNSON &amp; JOHNSON (XNYS:JNJ)</t>
+  </si>
+  <si>
+    <t>FEDEX CORPORATION (XNYS:FDX)</t>
+  </si>
+  <si>
+    <t>GENERAL ELECTRIC COMPANY (XNYS:GE)</t>
+  </si>
+  <si>
+    <t>LOCKHEED MARTIN CORPORATION (XNYS:LMT)</t>
+  </si>
+  <si>
     <t>Nyla Novak</t>
   </si>
   <si>
@@ -74,6 +160,27 @@
     <t>Mik Naam</t>
   </si>
   <si>
+    <t xml:space="preserve">     Bill SmITH</t>
+  </si>
+  <si>
+    <t>KEN Singh</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  Harley        Fritz</t>
+  </si>
+  <si>
+    <t>David    Rasmussen</t>
+  </si>
+  <si>
+    <t>IVAN HINEY</t>
+  </si>
+  <si>
+    <t>JONha Ma</t>
+  </si>
+  <si>
+    <t xml:space="preserve">     Jordan Boone</t>
+  </si>
+  <si>
     <t>Payment</t>
   </si>
   <si>
@@ -89,6 +196,54 @@
     <t>Transfer</t>
   </si>
   <si>
+    <t>BRENDAN Wallace</t>
+  </si>
+  <si>
+    <t xml:space="preserve">     Conor Wise</t>
+  </si>
+  <si>
+    <t>Steven     MIChael</t>
+  </si>
+  <si>
+    <t>JoSE   Roach</t>
+  </si>
+  <si>
+    <t>Franklin WRIGT</t>
+  </si>
+  <si>
+    <t xml:space="preserve">   Alia       Thornton</t>
+  </si>
+  <si>
+    <t>Denzel        Flores</t>
+  </si>
+  <si>
+    <t>Bruno CordOVA</t>
+  </si>
+  <si>
+    <t>jaylynn   napp</t>
+  </si>
+  <si>
+    <t>Bruce RICH</t>
+  </si>
+  <si>
+    <t xml:space="preserve">     Arturo Moore</t>
+  </si>
+  <si>
+    <t>Bryce     Carpenter</t>
+  </si>
+  <si>
+    <t>Jaidyn ANDERSEN</t>
+  </si>
+  <si>
+    <t>MARK WALM</t>
+  </si>
+  <si>
+    <t>HARRY LEE</t>
+  </si>
+  <si>
+    <t>JOSH JOHNSON</t>
+  </si>
+  <si>
     <t>Cloud Tech_Texas</t>
   </si>
   <si>
@@ -252,6 +407,610 @@
   </si>
   <si>
     <t>Josh Johnson</t>
+  </si>
+  <si>
+    <t>Region</t>
+  </si>
+  <si>
+    <t>Cloud Tech</t>
+  </si>
+  <si>
+    <t>Texas</t>
+  </si>
+  <si>
+    <t>Strategy</t>
+  </si>
+  <si>
+    <t>New York</t>
+  </si>
+  <si>
+    <t>Operations</t>
+  </si>
+  <si>
+    <t>Florida</t>
+  </si>
+  <si>
+    <t>Big Data</t>
+  </si>
+  <si>
+    <t>California</t>
+  </si>
+  <si>
+    <t>NA</t>
+  </si>
+  <si>
+    <t>Step</t>
+  </si>
+  <si>
+    <t>Transformation</t>
+  </si>
+  <si>
+    <t>Description</t>
+  </si>
+  <si>
+    <t>Formula / Shortcut</t>
+  </si>
+  <si>
+    <t>Autofit Rows &amp; Columns</t>
+  </si>
+  <si>
+    <t>Adjusted all row heights and column widths automatically so the dataset is fully visible and easier to read.</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Select entire table → </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Alt + H + O + I</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> (AutoFit Column Width) → </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Alt + H + O + A</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> (AutoFit Row Height)</t>
+    </r>
+  </si>
+  <si>
+    <t>Find &amp; Replace</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Removed unnecessary text enclosed in parentheses from the </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Client</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> column to standardize company names.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>Ctrl + H</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> → Find: </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>(*)</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> → Replace With: </t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>(blank)</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> → Replace All</t>
+    </r>
+  </si>
+  <si>
+    <t>Convert Text to Lowercase</t>
+  </si>
+  <si>
+    <t>Standardized all company names by converting them to lowercase for consistency. Created a temporary column, converted the text, pasted the results as values, and removed the original column.</t>
+  </si>
+  <si>
+    <r>
+      <t>=LOWER(original_cell)</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> → Copy → </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Paste Special → Values</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> → Delete original column</t>
+    </r>
+  </si>
+  <si>
+    <t>4</t>
+  </si>
+  <si>
+    <t>TRIM &amp; PROPER</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Cleaned the </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Contact</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> column by removing extra spaces and converting names to proper case (e.g., "Bill SmITH" → "Bill Smith"). Used a temporary column, pasted values, and removed the original column.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>=TRIM(PROPER(original_cell))</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> → Copy → </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Paste Special → Values</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> → Delete original column</t>
+    </r>
+  </si>
+  <si>
+    <t>5</t>
+  </si>
+  <si>
+    <t>Text to Columns</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Split the </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Department</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> column into two separate columns (</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Department</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> and </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Region</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>) using the underscore (</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>_</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>) delimiter.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Data → </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Text to Columns</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> → Delimited → Other: </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>_</t>
+    </r>
+  </si>
+  <si>
+    <t>Remove Duplicates</t>
+  </si>
+  <si>
+    <t>Removed duplicate records from the dataset to ensure each transaction appears only once.</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Select table → Data → </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Remove Duplicates</t>
+    </r>
+  </si>
+  <si>
+    <t>Fill Empty Cells</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Replaced all blank cells with </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>NA</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> to clearly indicate missing values and avoid confusion during analysis.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Home → Find &amp; Select → Go To Special → Blanks → Type </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>NA</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> → </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Ctrl + Enter</t>
+    </r>
+  </si>
+  <si>
+    <t>Handle Formula Errors</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Calculated </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Profit Margin</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> while preventing errors caused by missing Revenue or Profit values. If an error occurs, the formula returns </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>"NA"</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> instead of an Excel error.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>=IFERROR(Profit/Revenue,"NA")</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">(e.g., </t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>=IFERROR(I3/H3,"NA")</t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>)</t>
+    </r>
+  </si>
+  <si>
+    <t>9</t>
+  </si>
+  <si>
+    <t>Remove Gridlines</t>
+  </si>
+  <si>
+    <t>Hid worksheet gridlines to improve the visual presentation of the cleaned dataset.</t>
+  </si>
+  <si>
+    <t>Alt + W + V + G</t>
   </si>
 </sst>
 </file>
@@ -262,7 +1021,7 @@
     <numFmt numFmtId="6" formatCode="&quot;$&quot;#,##0_);[Red]\(&quot;$&quot;#,##0\)"/>
     <numFmt numFmtId="164" formatCode="0.0%"/>
   </numFmts>
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="7">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -277,16 +1036,56 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b/>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color theme="0"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="Arial Unicode MS"/>
+    </font>
+    <font>
+      <i/>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <i/>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="Arial Unicode MS"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -294,12 +1093,27 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="6" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -309,6 +1123,33 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="6" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -623,22 +1464,11 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FD37A31F-92F2-FA4A-B7ED-0F04A433817B}">
-  <dimension ref="B2:I42"/>
-  <sheetFormatPr defaultColWidth="11.19921875" defaultRowHeight="15.6" x14ac:dyDescent="0.3"/>
-  <cols>
-    <col min="1" max="1" width="6.69921875" customWidth="1"/>
-    <col min="2" max="2" width="9.5" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="42.5" customWidth="1"/>
-    <col min="4" max="4" width="17.19921875" customWidth="1"/>
-    <col min="5" max="5" width="17.19921875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="8.19921875" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="8.09765625" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="7" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="11.8984375" bestFit="1" customWidth="1"/>
-  </cols>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3CB85063-0D12-4852-B663-742E3D63B317}">
+  <dimension ref="B2:I33"/>
+  <sheetFormatPr defaultRowHeight="15.6"/>
   <sheetData>
-    <row r="2" spans="2:9" x14ac:dyDescent="0.3">
+    <row r="2" spans="2:9">
       <c r="B2" t="s">
         <v>0</v>
       </c>
@@ -652,7 +1482,7 @@
         <v>6</v>
       </c>
       <c r="F2" s="3" t="s">
-        <v>12</v>
+        <v>47</v>
       </c>
       <c r="G2" s="3" t="s">
         <v>2</v>
@@ -664,21 +1494,21 @@
         <v>4</v>
       </c>
     </row>
-    <row r="3" spans="2:9" x14ac:dyDescent="0.3">
+    <row r="3" spans="2:9">
       <c r="B3" s="4">
         <v>45076</v>
       </c>
       <c r="C3" t="s">
-        <v>21</v>
+        <v>7</v>
       </c>
       <c r="D3" t="s">
-        <v>49</v>
+        <v>40</v>
       </c>
       <c r="E3" t="s">
-        <v>17</v>
+        <v>68</v>
       </c>
       <c r="F3" t="s">
-        <v>16</v>
+        <v>51</v>
       </c>
       <c r="G3" s="1">
         <v>4500</v>
@@ -691,21 +1521,21 @@
         <v>0.13288888888888889</v>
       </c>
     </row>
-    <row r="4" spans="2:9" x14ac:dyDescent="0.3">
+    <row r="4" spans="2:9">
       <c r="B4" s="4">
         <v>45076</v>
       </c>
       <c r="C4" t="s">
-        <v>22</v>
+        <v>8</v>
       </c>
       <c r="D4" t="s">
-        <v>50</v>
+        <v>41</v>
       </c>
       <c r="E4" t="s">
-        <v>18</v>
+        <v>69</v>
       </c>
       <c r="F4" t="s">
-        <v>14</v>
+        <v>49</v>
       </c>
       <c r="G4" s="1">
         <v>3800</v>
@@ -714,22 +1544,22 @@
         <v>1045</v>
       </c>
       <c r="I4" s="2">
-        <f t="shared" ref="I4:I32" si="0">H4/G4</f>
+        <f t="shared" ref="I4:I33" si="0">H4/G4</f>
         <v>0.27500000000000002</v>
       </c>
     </row>
-    <row r="5" spans="2:9" x14ac:dyDescent="0.3">
+    <row r="5" spans="2:9">
       <c r="B5" s="4">
         <v>45076</v>
       </c>
       <c r="C5" t="s">
-        <v>23</v>
+        <v>9</v>
       </c>
       <c r="D5" t="s">
-        <v>51</v>
+        <v>42</v>
       </c>
       <c r="E5" t="s">
-        <v>18</v>
+        <v>69</v>
       </c>
       <c r="G5" s="1">
         <v>3712.5</v>
@@ -742,18 +1572,18 @@
         <v>0.2717845117845118</v>
       </c>
     </row>
-    <row r="6" spans="2:9" x14ac:dyDescent="0.3">
+    <row r="6" spans="2:9">
       <c r="B6" s="4">
         <v>45076</v>
       </c>
       <c r="C6" t="s">
-        <v>24</v>
+        <v>10</v>
       </c>
       <c r="D6" t="s">
-        <v>7</v>
+        <v>35</v>
       </c>
       <c r="E6" t="s">
-        <v>19</v>
+        <v>70</v>
       </c>
       <c r="G6" s="1"/>
       <c r="H6" s="1">
@@ -764,21 +1594,21 @@
         <v>#DIV/0!</v>
       </c>
     </row>
-    <row r="7" spans="2:9" x14ac:dyDescent="0.3">
+    <row r="7" spans="2:9">
       <c r="B7" s="4">
         <v>45076</v>
       </c>
       <c r="C7" t="s">
-        <v>25</v>
+        <v>11</v>
       </c>
       <c r="D7" t="s">
-        <v>52</v>
+        <v>43</v>
       </c>
       <c r="E7" t="s">
-        <v>19</v>
+        <v>70</v>
       </c>
       <c r="F7" t="s">
-        <v>15</v>
+        <v>50</v>
       </c>
       <c r="G7" s="1">
         <v>5000</v>
@@ -791,21 +1621,21 @@
         <v>0.1368</v>
       </c>
     </row>
-    <row r="8" spans="2:9" x14ac:dyDescent="0.3">
+    <row r="8" spans="2:9">
       <c r="B8" s="4">
         <v>45077</v>
       </c>
       <c r="C8" t="s">
-        <v>26</v>
+        <v>12</v>
       </c>
       <c r="D8" t="s">
-        <v>53</v>
+        <v>44</v>
       </c>
       <c r="E8" t="s">
-        <v>17</v>
+        <v>68</v>
       </c>
       <c r="F8" t="s">
-        <v>16</v>
+        <v>51</v>
       </c>
       <c r="G8" s="1">
         <v>6100</v>
@@ -818,21 +1648,21 @@
         <v>8.9180327868852466E-2</v>
       </c>
     </row>
-    <row r="9" spans="2:9" x14ac:dyDescent="0.3">
+    <row r="9" spans="2:9">
       <c r="B9" s="4">
         <v>45077</v>
       </c>
       <c r="C9" t="s">
-        <v>27</v>
+        <v>13</v>
       </c>
       <c r="D9" t="s">
-        <v>54</v>
+        <v>45</v>
       </c>
       <c r="E9" t="s">
-        <v>17</v>
+        <v>68</v>
       </c>
       <c r="F9" t="s">
-        <v>16</v>
+        <v>51</v>
       </c>
       <c r="G9" s="1">
         <v>4625</v>
@@ -845,21 +1675,21 @@
         <v>0.14486486486486486</v>
       </c>
     </row>
-    <row r="10" spans="2:9" x14ac:dyDescent="0.3">
+    <row r="10" spans="2:9">
       <c r="B10" s="4">
         <v>45077</v>
       </c>
       <c r="C10" t="s">
-        <v>28</v>
+        <v>14</v>
       </c>
       <c r="D10" t="s">
-        <v>55</v>
+        <v>46</v>
       </c>
       <c r="E10" t="s">
-        <v>17</v>
+        <v>68</v>
       </c>
       <c r="F10" t="s">
-        <v>16</v>
+        <v>51</v>
       </c>
       <c r="G10" s="1">
         <v>3800</v>
@@ -872,21 +1702,21 @@
         <v>0.53815789473684206</v>
       </c>
     </row>
-    <row r="11" spans="2:9" x14ac:dyDescent="0.3">
+    <row r="11" spans="2:9">
       <c r="B11" s="4">
         <v>45077</v>
       </c>
       <c r="C11" t="s">
-        <v>29</v>
+        <v>15</v>
       </c>
       <c r="D11" t="s">
-        <v>8</v>
+        <v>36</v>
       </c>
       <c r="E11" t="s">
-        <v>17</v>
+        <v>68</v>
       </c>
       <c r="F11" t="s">
-        <v>13</v>
+        <v>48</v>
       </c>
       <c r="G11" s="1">
         <v>3600</v>
@@ -899,21 +1729,21 @@
         <v>0.43444444444444447</v>
       </c>
     </row>
-    <row r="12" spans="2:9" x14ac:dyDescent="0.3">
+    <row r="12" spans="2:9">
       <c r="B12" s="4">
         <v>45077</v>
       </c>
       <c r="C12" t="s">
-        <v>30</v>
+        <v>16</v>
       </c>
       <c r="D12" t="s">
-        <v>9</v>
+        <v>37</v>
       </c>
       <c r="E12" t="s">
-        <v>17</v>
+        <v>68</v>
       </c>
       <c r="F12" t="s">
-        <v>15</v>
+        <v>50</v>
       </c>
       <c r="G12" s="1">
         <v>5100</v>
@@ -926,21 +1756,21 @@
         <v>0.23921568627450981</v>
       </c>
     </row>
-    <row r="13" spans="2:9" x14ac:dyDescent="0.3">
+    <row r="13" spans="2:9">
       <c r="B13" s="4">
         <v>45077</v>
       </c>
       <c r="C13" t="s">
-        <v>31</v>
+        <v>17</v>
       </c>
       <c r="D13" t="s">
-        <v>56</v>
+        <v>52</v>
       </c>
       <c r="E13" t="s">
-        <v>17</v>
+        <v>68</v>
       </c>
       <c r="F13" t="s">
-        <v>15</v>
+        <v>50</v>
       </c>
       <c r="G13" s="1">
         <v>4750</v>
@@ -953,21 +1783,21 @@
         <v>0.30210526315789471</v>
       </c>
     </row>
-    <row r="14" spans="2:9" x14ac:dyDescent="0.3">
+    <row r="14" spans="2:9">
       <c r="B14" s="4">
         <v>45077</v>
       </c>
       <c r="C14" t="s">
-        <v>32</v>
+        <v>18</v>
       </c>
       <c r="D14" t="s">
-        <v>57</v>
+        <v>53</v>
       </c>
       <c r="E14" t="s">
-        <v>19</v>
+        <v>70</v>
       </c>
       <c r="F14" t="s">
-        <v>16</v>
+        <v>51</v>
       </c>
       <c r="G14" s="1">
         <v>6000</v>
@@ -980,21 +1810,21 @@
         <v>0.16633333333333333</v>
       </c>
     </row>
-    <row r="15" spans="2:9" x14ac:dyDescent="0.3">
+    <row r="15" spans="2:9">
       <c r="B15" s="4">
         <v>45077</v>
       </c>
       <c r="C15" t="s">
-        <v>33</v>
+        <v>19</v>
       </c>
       <c r="D15" t="s">
-        <v>58</v>
+        <v>54</v>
       </c>
       <c r="E15" t="s">
-        <v>20</v>
+        <v>71</v>
       </c>
       <c r="F15" t="s">
-        <v>15</v>
+        <v>50</v>
       </c>
       <c r="G15" s="1">
         <v>4500</v>
@@ -1007,21 +1837,21 @@
         <v>0.17333333333333334</v>
       </c>
     </row>
-    <row r="16" spans="2:9" x14ac:dyDescent="0.3">
+    <row r="16" spans="2:9">
       <c r="B16" s="4">
         <v>45078</v>
       </c>
       <c r="C16" t="s">
-        <v>34</v>
+        <v>20</v>
       </c>
       <c r="D16" t="s">
-        <v>10</v>
+        <v>38</v>
       </c>
       <c r="E16" t="s">
-        <v>20</v>
+        <v>71</v>
       </c>
       <c r="F16" t="s">
-        <v>13</v>
+        <v>48</v>
       </c>
       <c r="G16" s="1"/>
       <c r="H16" s="1">
@@ -1032,21 +1862,21 @@
         <v>#DIV/0!</v>
       </c>
     </row>
-    <row r="17" spans="2:9" x14ac:dyDescent="0.3">
+    <row r="17" spans="2:9">
       <c r="B17" s="4">
         <v>45078</v>
       </c>
       <c r="C17" t="s">
-        <v>35</v>
+        <v>21</v>
       </c>
       <c r="D17" t="s">
-        <v>59</v>
+        <v>55</v>
       </c>
       <c r="E17" t="s">
-        <v>20</v>
+        <v>71</v>
       </c>
       <c r="F17" t="s">
-        <v>16</v>
+        <v>51</v>
       </c>
       <c r="G17" s="1">
         <v>3712.5</v>
@@ -1059,21 +1889,21 @@
         <v>0.32915824915824915</v>
       </c>
     </row>
-    <row r="18" spans="2:9" x14ac:dyDescent="0.3">
+    <row r="18" spans="2:9">
       <c r="B18" s="4">
         <v>45078</v>
       </c>
       <c r="C18" t="s">
-        <v>36</v>
+        <v>22</v>
       </c>
       <c r="D18" t="s">
-        <v>60</v>
+        <v>56</v>
       </c>
       <c r="E18" t="s">
-        <v>20</v>
+        <v>71</v>
       </c>
       <c r="F18" t="s">
-        <v>16</v>
+        <v>51</v>
       </c>
       <c r="G18" s="1">
         <v>4950</v>
@@ -1086,21 +1916,21 @@
         <v>0.21515151515151515</v>
       </c>
     </row>
-    <row r="19" spans="2:9" x14ac:dyDescent="0.3">
+    <row r="19" spans="2:9">
       <c r="B19" s="4">
         <v>45078</v>
       </c>
       <c r="C19" t="s">
-        <v>37</v>
+        <v>23</v>
       </c>
       <c r="D19" t="s">
-        <v>61</v>
+        <v>57</v>
       </c>
       <c r="E19" t="s">
-        <v>19</v>
+        <v>70</v>
       </c>
       <c r="F19" t="s">
-        <v>16</v>
+        <v>51</v>
       </c>
       <c r="G19" s="1">
         <v>4750</v>
@@ -1113,21 +1943,21 @@
         <v>0.17052631578947369</v>
       </c>
     </row>
-    <row r="20" spans="2:9" x14ac:dyDescent="0.3">
+    <row r="20" spans="2:9">
       <c r="B20" s="4">
         <v>45078</v>
       </c>
       <c r="C20" t="s">
-        <v>38</v>
+        <v>24</v>
       </c>
       <c r="D20" t="s">
-        <v>62</v>
+        <v>58</v>
       </c>
       <c r="E20" t="s">
-        <v>19</v>
+        <v>70</v>
       </c>
       <c r="F20" t="s">
-        <v>16</v>
+        <v>51</v>
       </c>
       <c r="G20" s="1">
         <v>7320</v>
@@ -1140,21 +1970,21 @@
         <v>0.12745901639344262</v>
       </c>
     </row>
-    <row r="21" spans="2:9" x14ac:dyDescent="0.3">
+    <row r="21" spans="2:9">
       <c r="B21" s="4">
         <v>45077</v>
       </c>
       <c r="C21" t="s">
-        <v>32</v>
+        <v>18</v>
       </c>
       <c r="D21" t="s">
-        <v>57</v>
+        <v>53</v>
       </c>
       <c r="E21" t="s">
-        <v>19</v>
+        <v>70</v>
       </c>
       <c r="F21" t="s">
-        <v>16</v>
+        <v>51</v>
       </c>
       <c r="G21" s="1">
         <v>6000</v>
@@ -1163,25 +1993,25 @@
         <v>998</v>
       </c>
       <c r="I21" s="2">
-        <f t="shared" ref="I21:I22" si="1">H21/G21</f>
+        <f t="shared" si="0"/>
         <v>0.16633333333333333</v>
       </c>
     </row>
-    <row r="22" spans="2:9" x14ac:dyDescent="0.3">
+    <row r="22" spans="2:9">
       <c r="B22" s="4">
         <v>45077</v>
       </c>
       <c r="C22" t="s">
-        <v>33</v>
+        <v>19</v>
       </c>
       <c r="D22" t="s">
-        <v>58</v>
+        <v>54</v>
       </c>
       <c r="E22" t="s">
-        <v>20</v>
+        <v>71</v>
       </c>
       <c r="F22" t="s">
-        <v>15</v>
+        <v>50</v>
       </c>
       <c r="G22" s="1">
         <v>4500</v>
@@ -1190,25 +2020,25 @@
         <v>780</v>
       </c>
       <c r="I22" s="2">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>0.17333333333333334</v>
       </c>
     </row>
-    <row r="23" spans="2:9" x14ac:dyDescent="0.3">
+    <row r="23" spans="2:9">
       <c r="B23" s="4">
         <v>45078</v>
       </c>
       <c r="C23" t="s">
-        <v>39</v>
+        <v>25</v>
       </c>
       <c r="D23" t="s">
-        <v>63</v>
+        <v>59</v>
       </c>
       <c r="E23" t="s">
-        <v>20</v>
+        <v>71</v>
       </c>
       <c r="F23" t="s">
-        <v>16</v>
+        <v>51</v>
       </c>
       <c r="G23" s="1">
         <v>5087.5</v>
@@ -1221,21 +2051,21 @@
         <v>0.12874692874692875</v>
       </c>
     </row>
-    <row r="24" spans="2:9" x14ac:dyDescent="0.3">
+    <row r="24" spans="2:9">
       <c r="B24" s="4">
         <v>45078</v>
       </c>
       <c r="C24" t="s">
-        <v>40</v>
+        <v>26</v>
       </c>
       <c r="D24" t="s">
-        <v>64</v>
+        <v>60</v>
       </c>
       <c r="E24" t="s">
-        <v>20</v>
+        <v>71</v>
       </c>
       <c r="F24" t="s">
-        <v>16</v>
+        <v>51</v>
       </c>
       <c r="G24" s="1">
         <v>4500</v>
@@ -1248,21 +2078,21 @@
         <v>0.16044444444444445</v>
       </c>
     </row>
-    <row r="25" spans="2:9" x14ac:dyDescent="0.3">
+    <row r="25" spans="2:9">
       <c r="B25" s="4">
         <v>45078</v>
       </c>
       <c r="C25" t="s">
-        <v>41</v>
+        <v>27</v>
       </c>
       <c r="D25" t="s">
-        <v>65</v>
+        <v>61</v>
       </c>
       <c r="E25" t="s">
-        <v>20</v>
+        <v>71</v>
       </c>
       <c r="F25" t="s">
-        <v>13</v>
+        <v>48</v>
       </c>
       <c r="G25" s="1">
         <v>4250</v>
@@ -1275,21 +2105,21 @@
         <v>0.21199999999999999</v>
       </c>
     </row>
-    <row r="26" spans="2:9" x14ac:dyDescent="0.3">
+    <row r="26" spans="2:9">
       <c r="B26" s="4">
         <v>45079</v>
       </c>
       <c r="C26" t="s">
-        <v>42</v>
+        <v>28</v>
       </c>
       <c r="D26" t="s">
-        <v>66</v>
+        <v>62</v>
       </c>
       <c r="E26" t="s">
-        <v>20</v>
+        <v>71</v>
       </c>
       <c r="F26" t="s">
-        <v>14</v>
+        <v>49</v>
       </c>
       <c r="G26" s="1">
         <v>5250</v>
@@ -1302,21 +2132,21 @@
         <v>0.25695238095238093</v>
       </c>
     </row>
-    <row r="27" spans="2:9" x14ac:dyDescent="0.3">
+    <row r="27" spans="2:9">
       <c r="B27" s="4">
         <v>45079</v>
       </c>
       <c r="C27" t="s">
-        <v>43</v>
+        <v>29</v>
       </c>
       <c r="D27" t="s">
-        <v>67</v>
+        <v>63</v>
       </c>
       <c r="E27" t="s">
-        <v>18</v>
+        <v>69</v>
       </c>
       <c r="F27" t="s">
-        <v>14</v>
+        <v>49</v>
       </c>
       <c r="G27" s="1">
         <v>6500</v>
@@ -1329,21 +2159,21 @@
         <v>0.19815384615384615</v>
       </c>
     </row>
-    <row r="28" spans="2:9" x14ac:dyDescent="0.3">
+    <row r="28" spans="2:9">
       <c r="B28" s="4">
         <v>45079</v>
       </c>
       <c r="C28" t="s">
-        <v>44</v>
+        <v>30</v>
       </c>
       <c r="D28" t="s">
-        <v>68</v>
+        <v>64</v>
       </c>
       <c r="E28" t="s">
-        <v>18</v>
+        <v>69</v>
       </c>
       <c r="F28" t="s">
-        <v>14</v>
+        <v>49</v>
       </c>
       <c r="G28" s="1">
         <v>7500</v>
@@ -1356,21 +2186,21 @@
         <v>0.22186666666666666</v>
       </c>
     </row>
-    <row r="29" spans="2:9" x14ac:dyDescent="0.3">
+    <row r="29" spans="2:9">
       <c r="B29" s="4">
         <v>45079</v>
       </c>
       <c r="C29" t="s">
-        <v>45</v>
+        <v>31</v>
       </c>
       <c r="D29" t="s">
+        <v>65</v>
+      </c>
+      <c r="E29" t="s">
         <v>69</v>
       </c>
-      <c r="E29" t="s">
-        <v>18</v>
-      </c>
       <c r="F29" t="s">
-        <v>16</v>
+        <v>51</v>
       </c>
       <c r="G29" s="1">
         <v>5500</v>
@@ -1383,21 +2213,21 @@
         <v>0.24</v>
       </c>
     </row>
-    <row r="30" spans="2:9" x14ac:dyDescent="0.3">
+    <row r="30" spans="2:9">
       <c r="B30" s="4">
         <v>45079</v>
       </c>
       <c r="C30" t="s">
-        <v>46</v>
+        <v>32</v>
       </c>
       <c r="D30" t="s">
-        <v>70</v>
+        <v>66</v>
       </c>
       <c r="E30" t="s">
-        <v>18</v>
+        <v>69</v>
       </c>
       <c r="F30" t="s">
-        <v>16</v>
+        <v>51</v>
       </c>
       <c r="G30" s="1">
         <v>4625</v>
@@ -1410,21 +2240,21 @@
         <v>0.21643243243243243</v>
       </c>
     </row>
-    <row r="31" spans="2:9" x14ac:dyDescent="0.3">
+    <row r="31" spans="2:9">
       <c r="B31" s="4">
         <v>45079</v>
       </c>
       <c r="C31" t="s">
-        <v>47</v>
+        <v>33</v>
       </c>
       <c r="D31" t="s">
-        <v>71</v>
+        <v>67</v>
       </c>
       <c r="E31" t="s">
-        <v>18</v>
+        <v>69</v>
       </c>
       <c r="F31" t="s">
-        <v>16</v>
+        <v>51</v>
       </c>
       <c r="G31" s="1">
         <v>4500</v>
@@ -1437,21 +2267,21 @@
         <v>0.21333333333333335</v>
       </c>
     </row>
-    <row r="32" spans="2:9" x14ac:dyDescent="0.3">
+    <row r="32" spans="2:9">
       <c r="B32" s="4">
         <v>45079</v>
       </c>
       <c r="C32" t="s">
+        <v>34</v>
+      </c>
+      <c r="D32" t="s">
+        <v>39</v>
+      </c>
+      <c r="E32" t="s">
+        <v>69</v>
+      </c>
+      <c r="F32" t="s">
         <v>48</v>
-      </c>
-      <c r="D32" t="s">
-        <v>11</v>
-      </c>
-      <c r="E32" t="s">
-        <v>18</v>
-      </c>
-      <c r="F32" t="s">
-        <v>13</v>
       </c>
       <c r="G32" s="1">
         <v>5400</v>
@@ -1464,21 +2294,21 @@
         <v>0.1</v>
       </c>
     </row>
-    <row r="33" spans="2:9" x14ac:dyDescent="0.3">
+    <row r="33" spans="2:9">
       <c r="B33" s="4">
         <v>45076</v>
       </c>
       <c r="C33" t="s">
-        <v>25</v>
+        <v>11</v>
       </c>
       <c r="D33" t="s">
-        <v>52</v>
+        <v>43</v>
       </c>
       <c r="E33" t="s">
-        <v>19</v>
+        <v>70</v>
       </c>
       <c r="F33" t="s">
-        <v>15</v>
+        <v>50</v>
       </c>
       <c r="G33" s="1">
         <v>5000</v>
@@ -1487,36 +2317,1085 @@
         <v>684</v>
       </c>
       <c r="I33" s="2">
-        <f t="shared" ref="I33" si="2">H33/G33</f>
+        <f t="shared" si="0"/>
         <v>0.1368</v>
       </c>
     </row>
-    <row r="34" spans="2:9" x14ac:dyDescent="0.3">
-      <c r="G34" s="1"/>
-    </row>
-    <row r="35" spans="2:9" x14ac:dyDescent="0.3">
-      <c r="G35" s="1"/>
-    </row>
-    <row r="36" spans="2:9" x14ac:dyDescent="0.3">
-      <c r="G36" s="1"/>
-    </row>
-    <row r="37" spans="2:9" x14ac:dyDescent="0.3">
-      <c r="G37" s="1"/>
-    </row>
-    <row r="38" spans="2:9" x14ac:dyDescent="0.3">
-      <c r="G38" s="1"/>
-    </row>
-    <row r="39" spans="2:9" x14ac:dyDescent="0.3">
-      <c r="G39" s="1"/>
-    </row>
-    <row r="40" spans="2:9" x14ac:dyDescent="0.3">
-      <c r="G40" s="1"/>
-    </row>
-    <row r="41" spans="2:9" x14ac:dyDescent="0.3">
-      <c r="G41" s="1"/>
-    </row>
-    <row r="42" spans="2:9" x14ac:dyDescent="0.3">
-      <c r="G42" s="1"/>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FD37A31F-92F2-FA4A-B7ED-0F04A433817B}">
+  <dimension ref="B2:J42"/>
+  <sheetFormatPr defaultColWidth="11.19921875" defaultRowHeight="15.6"/>
+  <cols>
+    <col min="1" max="1" width="6.69921875" style="3" customWidth="1"/>
+    <col min="2" max="2" width="9.5" style="3" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="42.5" style="3" customWidth="1"/>
+    <col min="4" max="4" width="17.19921875" style="3" customWidth="1"/>
+    <col min="5" max="5" width="17.19921875" style="3" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="17.19921875" style="3" customWidth="1"/>
+    <col min="7" max="7" width="8.19921875" style="3" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="8.09765625" style="3" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="7" style="3" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="11.8984375" style="3" bestFit="1" customWidth="1"/>
+    <col min="11" max="16384" width="11.19921875" style="3"/>
+  </cols>
+  <sheetData>
+    <row r="2" spans="2:10">
+      <c r="B2" s="5" t="s">
+        <v>0</v>
+      </c>
+      <c r="C2" s="5" t="s">
+        <v>5</v>
+      </c>
+      <c r="D2" s="5" t="s">
+        <v>1</v>
+      </c>
+      <c r="E2" s="5" t="s">
+        <v>6</v>
+      </c>
+      <c r="F2" s="5" t="s">
+        <v>123</v>
+      </c>
+      <c r="G2" s="5" t="s">
+        <v>47</v>
+      </c>
+      <c r="H2" s="5" t="s">
+        <v>2</v>
+      </c>
+      <c r="I2" s="5" t="s">
+        <v>3</v>
+      </c>
+      <c r="J2" s="5" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="3" spans="2:10">
+      <c r="B3" s="6">
+        <v>45076</v>
+      </c>
+      <c r="C3" s="7" t="s">
+        <v>72</v>
+      </c>
+      <c r="D3" s="7" t="s">
+        <v>100</v>
+      </c>
+      <c r="E3" s="7" t="s">
+        <v>124</v>
+      </c>
+      <c r="F3" s="7" t="s">
+        <v>125</v>
+      </c>
+      <c r="G3" s="7" t="s">
+        <v>51</v>
+      </c>
+      <c r="H3" s="8">
+        <v>4500</v>
+      </c>
+      <c r="I3" s="8">
+        <v>598</v>
+      </c>
+      <c r="J3" s="9">
+        <f>IFERROR(I3/H3,"NA")</f>
+        <v>0.13288888888888889</v>
+      </c>
+    </row>
+    <row r="4" spans="2:10">
+      <c r="B4" s="6">
+        <v>45076</v>
+      </c>
+      <c r="C4" s="7" t="s">
+        <v>73</v>
+      </c>
+      <c r="D4" s="7" t="s">
+        <v>101</v>
+      </c>
+      <c r="E4" s="7" t="s">
+        <v>126</v>
+      </c>
+      <c r="F4" s="7" t="s">
+        <v>127</v>
+      </c>
+      <c r="G4" s="7" t="s">
+        <v>49</v>
+      </c>
+      <c r="H4" s="8">
+        <v>3800</v>
+      </c>
+      <c r="I4" s="8">
+        <v>1045</v>
+      </c>
+      <c r="J4" s="9">
+        <f t="shared" ref="J4:J30" si="0">IFERROR(I4/H4,"NA")</f>
+        <v>0.27500000000000002</v>
+      </c>
+    </row>
+    <row r="5" spans="2:10">
+      <c r="B5" s="6">
+        <v>45076</v>
+      </c>
+      <c r="C5" s="7" t="s">
+        <v>74</v>
+      </c>
+      <c r="D5" s="7" t="s">
+        <v>102</v>
+      </c>
+      <c r="E5" s="7" t="s">
+        <v>126</v>
+      </c>
+      <c r="F5" s="7" t="s">
+        <v>127</v>
+      </c>
+      <c r="G5" s="7" t="s">
+        <v>132</v>
+      </c>
+      <c r="H5" s="8">
+        <v>3712.5</v>
+      </c>
+      <c r="I5" s="8">
+        <v>1009</v>
+      </c>
+      <c r="J5" s="9">
+        <f t="shared" si="0"/>
+        <v>0.2717845117845118</v>
+      </c>
+    </row>
+    <row r="6" spans="2:10">
+      <c r="B6" s="6">
+        <v>45076</v>
+      </c>
+      <c r="C6" s="7" t="s">
+        <v>75</v>
+      </c>
+      <c r="D6" s="7" t="s">
+        <v>35</v>
+      </c>
+      <c r="E6" s="7" t="s">
+        <v>128</v>
+      </c>
+      <c r="F6" s="7" t="s">
+        <v>129</v>
+      </c>
+      <c r="G6" s="7" t="s">
+        <v>132</v>
+      </c>
+      <c r="H6" s="8" t="s">
+        <v>132</v>
+      </c>
+      <c r="I6" s="8">
+        <v>779</v>
+      </c>
+      <c r="J6" s="9" t="str">
+        <f t="shared" si="0"/>
+        <v>NA</v>
+      </c>
+    </row>
+    <row r="7" spans="2:10">
+      <c r="B7" s="6">
+        <v>45076</v>
+      </c>
+      <c r="C7" s="7" t="s">
+        <v>76</v>
+      </c>
+      <c r="D7" s="7" t="s">
+        <v>103</v>
+      </c>
+      <c r="E7" s="7" t="s">
+        <v>128</v>
+      </c>
+      <c r="F7" s="7" t="s">
+        <v>129</v>
+      </c>
+      <c r="G7" s="7" t="s">
+        <v>50</v>
+      </c>
+      <c r="H7" s="8">
+        <v>5000</v>
+      </c>
+      <c r="I7" s="8">
+        <v>684</v>
+      </c>
+      <c r="J7" s="9">
+        <f t="shared" si="0"/>
+        <v>0.1368</v>
+      </c>
+    </row>
+    <row r="8" spans="2:10">
+      <c r="B8" s="6">
+        <v>45077</v>
+      </c>
+      <c r="C8" s="7" t="s">
+        <v>77</v>
+      </c>
+      <c r="D8" s="7" t="s">
+        <v>104</v>
+      </c>
+      <c r="E8" s="7" t="s">
+        <v>124</v>
+      </c>
+      <c r="F8" s="7" t="s">
+        <v>125</v>
+      </c>
+      <c r="G8" s="7" t="s">
+        <v>51</v>
+      </c>
+      <c r="H8" s="8">
+        <v>6100</v>
+      </c>
+      <c r="I8" s="8">
+        <v>544</v>
+      </c>
+      <c r="J8" s="9">
+        <f t="shared" si="0"/>
+        <v>8.9180327868852466E-2</v>
+      </c>
+    </row>
+    <row r="9" spans="2:10">
+      <c r="B9" s="6">
+        <v>45077</v>
+      </c>
+      <c r="C9" s="7" t="s">
+        <v>78</v>
+      </c>
+      <c r="D9" s="7" t="s">
+        <v>105</v>
+      </c>
+      <c r="E9" s="7" t="s">
+        <v>124</v>
+      </c>
+      <c r="F9" s="7" t="s">
+        <v>125</v>
+      </c>
+      <c r="G9" s="7" t="s">
+        <v>51</v>
+      </c>
+      <c r="H9" s="8">
+        <v>4625</v>
+      </c>
+      <c r="I9" s="8">
+        <v>670</v>
+      </c>
+      <c r="J9" s="9">
+        <f t="shared" si="0"/>
+        <v>0.14486486486486486</v>
+      </c>
+    </row>
+    <row r="10" spans="2:10">
+      <c r="B10" s="6">
+        <v>45077</v>
+      </c>
+      <c r="C10" s="7" t="s">
+        <v>79</v>
+      </c>
+      <c r="D10" s="7" t="s">
+        <v>106</v>
+      </c>
+      <c r="E10" s="7" t="s">
+        <v>124</v>
+      </c>
+      <c r="F10" s="7" t="s">
+        <v>125</v>
+      </c>
+      <c r="G10" s="7" t="s">
+        <v>51</v>
+      </c>
+      <c r="H10" s="8">
+        <v>3800</v>
+      </c>
+      <c r="I10" s="8">
+        <v>2045</v>
+      </c>
+      <c r="J10" s="9">
+        <f t="shared" si="0"/>
+        <v>0.53815789473684206</v>
+      </c>
+    </row>
+    <row r="11" spans="2:10">
+      <c r="B11" s="6">
+        <v>45077</v>
+      </c>
+      <c r="C11" s="7" t="s">
+        <v>80</v>
+      </c>
+      <c r="D11" s="7" t="s">
+        <v>36</v>
+      </c>
+      <c r="E11" s="7" t="s">
+        <v>124</v>
+      </c>
+      <c r="F11" s="7" t="s">
+        <v>125</v>
+      </c>
+      <c r="G11" s="7" t="s">
+        <v>48</v>
+      </c>
+      <c r="H11" s="8">
+        <v>3600</v>
+      </c>
+      <c r="I11" s="8">
+        <v>1564</v>
+      </c>
+      <c r="J11" s="9">
+        <f t="shared" si="0"/>
+        <v>0.43444444444444447</v>
+      </c>
+    </row>
+    <row r="12" spans="2:10">
+      <c r="B12" s="6">
+        <v>45077</v>
+      </c>
+      <c r="C12" s="7" t="s">
+        <v>81</v>
+      </c>
+      <c r="D12" s="7" t="s">
+        <v>37</v>
+      </c>
+      <c r="E12" s="7" t="s">
+        <v>124</v>
+      </c>
+      <c r="F12" s="7" t="s">
+        <v>125</v>
+      </c>
+      <c r="G12" s="7" t="s">
+        <v>50</v>
+      </c>
+      <c r="H12" s="8">
+        <v>5100</v>
+      </c>
+      <c r="I12" s="8">
+        <v>1220</v>
+      </c>
+      <c r="J12" s="9">
+        <f t="shared" si="0"/>
+        <v>0.23921568627450981</v>
+      </c>
+    </row>
+    <row r="13" spans="2:10">
+      <c r="B13" s="6">
+        <v>45077</v>
+      </c>
+      <c r="C13" s="7" t="s">
+        <v>82</v>
+      </c>
+      <c r="D13" s="7" t="s">
+        <v>107</v>
+      </c>
+      <c r="E13" s="7" t="s">
+        <v>124</v>
+      </c>
+      <c r="F13" s="7" t="s">
+        <v>125</v>
+      </c>
+      <c r="G13" s="7" t="s">
+        <v>50</v>
+      </c>
+      <c r="H13" s="8">
+        <v>4750</v>
+      </c>
+      <c r="I13" s="8">
+        <v>1435</v>
+      </c>
+      <c r="J13" s="9">
+        <f t="shared" si="0"/>
+        <v>0.30210526315789471</v>
+      </c>
+    </row>
+    <row r="14" spans="2:10">
+      <c r="B14" s="6">
+        <v>45077</v>
+      </c>
+      <c r="C14" s="7" t="s">
+        <v>83</v>
+      </c>
+      <c r="D14" s="7" t="s">
+        <v>108</v>
+      </c>
+      <c r="E14" s="7" t="s">
+        <v>128</v>
+      </c>
+      <c r="F14" s="7" t="s">
+        <v>129</v>
+      </c>
+      <c r="G14" s="7" t="s">
+        <v>51</v>
+      </c>
+      <c r="H14" s="8">
+        <v>6000</v>
+      </c>
+      <c r="I14" s="8">
+        <v>998</v>
+      </c>
+      <c r="J14" s="9">
+        <f t="shared" si="0"/>
+        <v>0.16633333333333333</v>
+      </c>
+    </row>
+    <row r="15" spans="2:10">
+      <c r="B15" s="6">
+        <v>45077</v>
+      </c>
+      <c r="C15" s="7" t="s">
+        <v>84</v>
+      </c>
+      <c r="D15" s="7" t="s">
+        <v>109</v>
+      </c>
+      <c r="E15" s="7" t="s">
+        <v>130</v>
+      </c>
+      <c r="F15" s="7" t="s">
+        <v>131</v>
+      </c>
+      <c r="G15" s="7" t="s">
+        <v>50</v>
+      </c>
+      <c r="H15" s="8">
+        <v>4500</v>
+      </c>
+      <c r="I15" s="8">
+        <v>780</v>
+      </c>
+      <c r="J15" s="9">
+        <f t="shared" si="0"/>
+        <v>0.17333333333333334</v>
+      </c>
+    </row>
+    <row r="16" spans="2:10">
+      <c r="B16" s="6">
+        <v>45078</v>
+      </c>
+      <c r="C16" s="7" t="s">
+        <v>85</v>
+      </c>
+      <c r="D16" s="7" t="s">
+        <v>38</v>
+      </c>
+      <c r="E16" s="7" t="s">
+        <v>130</v>
+      </c>
+      <c r="F16" s="7" t="s">
+        <v>131</v>
+      </c>
+      <c r="G16" s="7" t="s">
+        <v>48</v>
+      </c>
+      <c r="H16" s="8" t="s">
+        <v>132</v>
+      </c>
+      <c r="I16" s="8">
+        <v>1044</v>
+      </c>
+      <c r="J16" s="9" t="str">
+        <f t="shared" si="0"/>
+        <v>NA</v>
+      </c>
+    </row>
+    <row r="17" spans="2:10">
+      <c r="B17" s="6">
+        <v>45078</v>
+      </c>
+      <c r="C17" s="7" t="s">
+        <v>86</v>
+      </c>
+      <c r="D17" s="7" t="s">
+        <v>110</v>
+      </c>
+      <c r="E17" s="7" t="s">
+        <v>130</v>
+      </c>
+      <c r="F17" s="7" t="s">
+        <v>131</v>
+      </c>
+      <c r="G17" s="7" t="s">
+        <v>51</v>
+      </c>
+      <c r="H17" s="8">
+        <v>3712.5</v>
+      </c>
+      <c r="I17" s="8">
+        <v>1222</v>
+      </c>
+      <c r="J17" s="9">
+        <f t="shared" si="0"/>
+        <v>0.32915824915824915</v>
+      </c>
+    </row>
+    <row r="18" spans="2:10">
+      <c r="B18" s="6">
+        <v>45078</v>
+      </c>
+      <c r="C18" s="7" t="s">
+        <v>87</v>
+      </c>
+      <c r="D18" s="7" t="s">
+        <v>111</v>
+      </c>
+      <c r="E18" s="7" t="s">
+        <v>130</v>
+      </c>
+      <c r="F18" s="7" t="s">
+        <v>131</v>
+      </c>
+      <c r="G18" s="7" t="s">
+        <v>51</v>
+      </c>
+      <c r="H18" s="8">
+        <v>4950</v>
+      </c>
+      <c r="I18" s="8">
+        <v>1065</v>
+      </c>
+      <c r="J18" s="9">
+        <f t="shared" si="0"/>
+        <v>0.21515151515151515</v>
+      </c>
+    </row>
+    <row r="19" spans="2:10">
+      <c r="B19" s="6">
+        <v>45078</v>
+      </c>
+      <c r="C19" s="7" t="s">
+        <v>88</v>
+      </c>
+      <c r="D19" s="7" t="s">
+        <v>112</v>
+      </c>
+      <c r="E19" s="7" t="s">
+        <v>128</v>
+      </c>
+      <c r="F19" s="7" t="s">
+        <v>129</v>
+      </c>
+      <c r="G19" s="7" t="s">
+        <v>51</v>
+      </c>
+      <c r="H19" s="8">
+        <v>4750</v>
+      </c>
+      <c r="I19" s="8">
+        <v>810</v>
+      </c>
+      <c r="J19" s="9">
+        <f t="shared" si="0"/>
+        <v>0.17052631578947369</v>
+      </c>
+    </row>
+    <row r="20" spans="2:10">
+      <c r="B20" s="6">
+        <v>45078</v>
+      </c>
+      <c r="C20" s="7" t="s">
+        <v>89</v>
+      </c>
+      <c r="D20" s="7" t="s">
+        <v>113</v>
+      </c>
+      <c r="E20" s="7" t="s">
+        <v>128</v>
+      </c>
+      <c r="F20" s="7" t="s">
+        <v>129</v>
+      </c>
+      <c r="G20" s="7" t="s">
+        <v>51</v>
+      </c>
+      <c r="H20" s="8">
+        <v>7320</v>
+      </c>
+      <c r="I20" s="8">
+        <v>933</v>
+      </c>
+      <c r="J20" s="9">
+        <f t="shared" si="0"/>
+        <v>0.12745901639344262</v>
+      </c>
+    </row>
+    <row r="21" spans="2:10">
+      <c r="B21" s="6">
+        <v>45078</v>
+      </c>
+      <c r="C21" s="7" t="s">
+        <v>90</v>
+      </c>
+      <c r="D21" s="7" t="s">
+        <v>114</v>
+      </c>
+      <c r="E21" s="7" t="s">
+        <v>130</v>
+      </c>
+      <c r="F21" s="7" t="s">
+        <v>131</v>
+      </c>
+      <c r="G21" s="7" t="s">
+        <v>51</v>
+      </c>
+      <c r="H21" s="8">
+        <v>5087.5</v>
+      </c>
+      <c r="I21" s="8">
+        <v>655</v>
+      </c>
+      <c r="J21" s="9">
+        <f t="shared" si="0"/>
+        <v>0.12874692874692875</v>
+      </c>
+    </row>
+    <row r="22" spans="2:10">
+      <c r="B22" s="6">
+        <v>45078</v>
+      </c>
+      <c r="C22" s="7" t="s">
+        <v>91</v>
+      </c>
+      <c r="D22" s="7" t="s">
+        <v>115</v>
+      </c>
+      <c r="E22" s="7" t="s">
+        <v>130</v>
+      </c>
+      <c r="F22" s="7" t="s">
+        <v>131</v>
+      </c>
+      <c r="G22" s="7" t="s">
+        <v>51</v>
+      </c>
+      <c r="H22" s="8">
+        <v>4500</v>
+      </c>
+      <c r="I22" s="8">
+        <v>722</v>
+      </c>
+      <c r="J22" s="9">
+        <f t="shared" si="0"/>
+        <v>0.16044444444444445</v>
+      </c>
+    </row>
+    <row r="23" spans="2:10">
+      <c r="B23" s="6">
+        <v>45078</v>
+      </c>
+      <c r="C23" s="7" t="s">
+        <v>92</v>
+      </c>
+      <c r="D23" s="7" t="s">
+        <v>116</v>
+      </c>
+      <c r="E23" s="7" t="s">
+        <v>130</v>
+      </c>
+      <c r="F23" s="7" t="s">
+        <v>131</v>
+      </c>
+      <c r="G23" s="7" t="s">
+        <v>48</v>
+      </c>
+      <c r="H23" s="8">
+        <v>4250</v>
+      </c>
+      <c r="I23" s="8">
+        <v>901</v>
+      </c>
+      <c r="J23" s="9">
+        <f t="shared" si="0"/>
+        <v>0.21199999999999999</v>
+      </c>
+    </row>
+    <row r="24" spans="2:10">
+      <c r="B24" s="6">
+        <v>45079</v>
+      </c>
+      <c r="C24" s="7" t="s">
+        <v>93</v>
+      </c>
+      <c r="D24" s="7" t="s">
+        <v>117</v>
+      </c>
+      <c r="E24" s="7" t="s">
+        <v>130</v>
+      </c>
+      <c r="F24" s="7" t="s">
+        <v>131</v>
+      </c>
+      <c r="G24" s="7" t="s">
+        <v>49</v>
+      </c>
+      <c r="H24" s="8">
+        <v>5250</v>
+      </c>
+      <c r="I24" s="8">
+        <v>1349</v>
+      </c>
+      <c r="J24" s="9">
+        <f t="shared" si="0"/>
+        <v>0.25695238095238093</v>
+      </c>
+    </row>
+    <row r="25" spans="2:10">
+      <c r="B25" s="6">
+        <v>45079</v>
+      </c>
+      <c r="C25" s="7" t="s">
+        <v>94</v>
+      </c>
+      <c r="D25" s="7" t="s">
+        <v>118</v>
+      </c>
+      <c r="E25" s="7" t="s">
+        <v>126</v>
+      </c>
+      <c r="F25" s="7" t="s">
+        <v>127</v>
+      </c>
+      <c r="G25" s="7" t="s">
+        <v>49</v>
+      </c>
+      <c r="H25" s="8">
+        <v>6500</v>
+      </c>
+      <c r="I25" s="8">
+        <v>1288</v>
+      </c>
+      <c r="J25" s="9">
+        <f t="shared" si="0"/>
+        <v>0.19815384615384615</v>
+      </c>
+    </row>
+    <row r="26" spans="2:10">
+      <c r="B26" s="6">
+        <v>45079</v>
+      </c>
+      <c r="C26" s="7" t="s">
+        <v>95</v>
+      </c>
+      <c r="D26" s="7" t="s">
+        <v>119</v>
+      </c>
+      <c r="E26" s="7" t="s">
+        <v>126</v>
+      </c>
+      <c r="F26" s="7" t="s">
+        <v>127</v>
+      </c>
+      <c r="G26" s="7" t="s">
+        <v>49</v>
+      </c>
+      <c r="H26" s="8">
+        <v>7500</v>
+      </c>
+      <c r="I26" s="8">
+        <v>1664</v>
+      </c>
+      <c r="J26" s="9">
+        <f t="shared" si="0"/>
+        <v>0.22186666666666666</v>
+      </c>
+    </row>
+    <row r="27" spans="2:10">
+      <c r="B27" s="6">
+        <v>45079</v>
+      </c>
+      <c r="C27" s="7" t="s">
+        <v>96</v>
+      </c>
+      <c r="D27" s="7" t="s">
+        <v>120</v>
+      </c>
+      <c r="E27" s="7" t="s">
+        <v>126</v>
+      </c>
+      <c r="F27" s="7" t="s">
+        <v>127</v>
+      </c>
+      <c r="G27" s="7" t="s">
+        <v>51</v>
+      </c>
+      <c r="H27" s="8">
+        <v>5500</v>
+      </c>
+      <c r="I27" s="8">
+        <v>1320</v>
+      </c>
+      <c r="J27" s="9">
+        <f t="shared" si="0"/>
+        <v>0.24</v>
+      </c>
+    </row>
+    <row r="28" spans="2:10">
+      <c r="B28" s="6">
+        <v>45079</v>
+      </c>
+      <c r="C28" s="7" t="s">
+        <v>97</v>
+      </c>
+      <c r="D28" s="7" t="s">
+        <v>121</v>
+      </c>
+      <c r="E28" s="7" t="s">
+        <v>126</v>
+      </c>
+      <c r="F28" s="7" t="s">
+        <v>127</v>
+      </c>
+      <c r="G28" s="7" t="s">
+        <v>51</v>
+      </c>
+      <c r="H28" s="8">
+        <v>4625</v>
+      </c>
+      <c r="I28" s="8">
+        <v>1001</v>
+      </c>
+      <c r="J28" s="9">
+        <f t="shared" si="0"/>
+        <v>0.21643243243243243</v>
+      </c>
+    </row>
+    <row r="29" spans="2:10">
+      <c r="B29" s="6">
+        <v>45079</v>
+      </c>
+      <c r="C29" s="7" t="s">
+        <v>98</v>
+      </c>
+      <c r="D29" s="7" t="s">
+        <v>122</v>
+      </c>
+      <c r="E29" s="7" t="s">
+        <v>126</v>
+      </c>
+      <c r="F29" s="7" t="s">
+        <v>127</v>
+      </c>
+      <c r="G29" s="7" t="s">
+        <v>51</v>
+      </c>
+      <c r="H29" s="8">
+        <v>4500</v>
+      </c>
+      <c r="I29" s="8">
+        <v>960</v>
+      </c>
+      <c r="J29" s="9">
+        <f t="shared" si="0"/>
+        <v>0.21333333333333335</v>
+      </c>
+    </row>
+    <row r="30" spans="2:10">
+      <c r="B30" s="6">
+        <v>45079</v>
+      </c>
+      <c r="C30" s="7" t="s">
+        <v>99</v>
+      </c>
+      <c r="D30" s="7" t="s">
+        <v>39</v>
+      </c>
+      <c r="E30" s="7" t="s">
+        <v>126</v>
+      </c>
+      <c r="F30" s="7" t="s">
+        <v>127</v>
+      </c>
+      <c r="G30" s="7" t="s">
+        <v>48</v>
+      </c>
+      <c r="H30" s="8">
+        <v>5400</v>
+      </c>
+      <c r="I30" s="8">
+        <v>540</v>
+      </c>
+      <c r="J30" s="9">
+        <f t="shared" si="0"/>
+        <v>0.1</v>
+      </c>
+    </row>
+    <row r="34" spans="8:8">
+      <c r="H34" s="1"/>
+    </row>
+    <row r="35" spans="8:8">
+      <c r="H35" s="1"/>
+    </row>
+    <row r="36" spans="8:8">
+      <c r="H36" s="1"/>
+    </row>
+    <row r="37" spans="8:8">
+      <c r="H37" s="1"/>
+    </row>
+    <row r="38" spans="8:8">
+      <c r="H38" s="1"/>
+    </row>
+    <row r="39" spans="8:8">
+      <c r="H39" s="1"/>
+    </row>
+    <row r="40" spans="8:8">
+      <c r="H40" s="1"/>
+    </row>
+    <row r="41" spans="8:8">
+      <c r="H41" s="1"/>
+    </row>
+    <row r="42" spans="8:8">
+      <c r="H42" s="1"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D5D74BC0-CB02-4A7D-9264-F0EA2C662565}">
+  <dimension ref="B3:E12"/>
+  <sheetFormatPr defaultRowHeight="15.6"/>
+  <cols>
+    <col min="2" max="2" width="4.59765625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="16.8984375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="20.3984375" customWidth="1"/>
+    <col min="5" max="5" width="20.19921875" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="3" spans="2:5">
+      <c r="B3" s="10" t="s">
+        <v>133</v>
+      </c>
+      <c r="C3" s="10" t="s">
+        <v>134</v>
+      </c>
+      <c r="D3" s="10" t="s">
+        <v>135</v>
+      </c>
+      <c r="E3" s="10" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="4" spans="2:5" ht="93.6">
+      <c r="B4" s="11">
+        <v>1</v>
+      </c>
+      <c r="C4" s="11" t="s">
+        <v>137</v>
+      </c>
+      <c r="D4" s="11" t="s">
+        <v>138</v>
+      </c>
+      <c r="E4" s="11" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="5" spans="2:5" ht="93.6">
+      <c r="B5" s="11">
+        <v>2</v>
+      </c>
+      <c r="C5" s="11" t="s">
+        <v>140</v>
+      </c>
+      <c r="D5" s="11" t="s">
+        <v>141</v>
+      </c>
+      <c r="E5" s="12" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="6" spans="2:5" ht="156">
+      <c r="B6" s="11">
+        <v>3</v>
+      </c>
+      <c r="C6" s="11" t="s">
+        <v>143</v>
+      </c>
+      <c r="D6" s="11" t="s">
+        <v>144</v>
+      </c>
+      <c r="E6" s="13" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="7" spans="2:5" ht="171.6">
+      <c r="B7" s="11" t="s">
+        <v>146</v>
+      </c>
+      <c r="C7" s="11" t="s">
+        <v>147</v>
+      </c>
+      <c r="D7" s="11" t="s">
+        <v>148</v>
+      </c>
+      <c r="E7" s="13" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="8" spans="2:5" ht="109.2">
+      <c r="B8" s="11" t="s">
+        <v>150</v>
+      </c>
+      <c r="C8" s="11" t="s">
+        <v>151</v>
+      </c>
+      <c r="D8" s="11" t="s">
+        <v>152</v>
+      </c>
+      <c r="E8" s="11" t="s">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="9" spans="2:5" ht="78">
+      <c r="B9" s="11">
+        <v>6</v>
+      </c>
+      <c r="C9" s="11" t="s">
+        <v>154</v>
+      </c>
+      <c r="D9" s="11" t="s">
+        <v>155</v>
+      </c>
+      <c r="E9" s="11" t="s">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="10" spans="2:5" ht="78">
+      <c r="B10" s="11">
+        <v>7</v>
+      </c>
+      <c r="C10" s="11" t="s">
+        <v>157</v>
+      </c>
+      <c r="D10" s="11" t="s">
+        <v>158</v>
+      </c>
+      <c r="E10" s="11" t="s">
+        <v>159</v>
+      </c>
+    </row>
+    <row r="11" spans="2:5" ht="140.4">
+      <c r="B11" s="11">
+        <v>8</v>
+      </c>
+      <c r="C11" s="11" t="s">
+        <v>160</v>
+      </c>
+      <c r="D11" s="11" t="s">
+        <v>161</v>
+      </c>
+      <c r="E11" s="13" t="s">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="12" spans="2:5" ht="78">
+      <c r="B12" s="11" t="s">
+        <v>163</v>
+      </c>
+      <c r="C12" s="11" t="s">
+        <v>164</v>
+      </c>
+      <c r="D12" s="11" t="s">
+        <v>165</v>
+      </c>
+      <c r="E12" s="12" t="s">
+        <v>166</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>